<commit_message>
rename directories, update BOM file, cleanup unnecessary files
</commit_message>
<xml_diff>
--- a/CM5IO_BOM.xlsx
+++ b/CM5IO_BOM.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Elektronika Schematy\KiCad\IARC-RPi_CM5_drone_platform\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67D9C42B-4691-4DFF-8C0A-2C4A4DFB5171}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD108B92-E698-4CEB-89CB-2782784DAF2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" activeTab="2" xr2:uid="{2D0DF511-CD42-495F-98C8-D8FF06CCC30B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" activeTab="4" xr2:uid="{2D0DF511-CD42-495F-98C8-D8FF06CCC30B}"/>
   </bookViews>
   <sheets>
     <sheet name="Bottom" sheetId="1" r:id="rId1"/>
     <sheet name="Top" sheetId="3" r:id="rId2"/>
     <sheet name="TME ZAMÓWIENIE" sheetId="7" r:id="rId3"/>
     <sheet name="MOUSER ZAMÓWIENIE" sheetId="4" r:id="rId4"/>
+    <sheet name="Mouser zamówienie dodatkowe" sheetId="8" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -61,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="274">
   <si>
     <t>Ilość</t>
   </si>
@@ -817,6 +818,72 @@
   </si>
   <si>
     <t>Koszt</t>
+  </si>
+  <si>
+    <t>Mistake has been made here - this is 10uF instead of 100uF. Soldered anyway.</t>
+  </si>
+  <si>
+    <t>10nF was not available. Soldered from private stash.</t>
+  </si>
+  <si>
+    <t>Here also is a mistake - should be 10uF, is 1uF. Soldered from private stash.</t>
+  </si>
+  <si>
+    <t>CM5 Dev board</t>
+  </si>
+  <si>
+    <t>Kabel Micro HDMI</t>
+  </si>
+  <si>
+    <t>Złącza Micro HDMI</t>
+  </si>
+  <si>
+    <t>Złącza ZIF do MIPI</t>
+  </si>
+  <si>
+    <t>Tantale pod USB - KEMET D 100uF</t>
+  </si>
+  <si>
+    <t>Ilość po uwzględnieniu progów cenowych</t>
+  </si>
+  <si>
+    <t>Ilość docelowa</t>
+  </si>
+  <si>
+    <t>USB A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">358-SC0358 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">538-46765-0301 </t>
+  </si>
+  <si>
+    <t>Nr prod MOUSER</t>
+  </si>
+  <si>
+    <t>&lt;-</t>
+  </si>
+  <si>
+    <t>TYLE OSTATECZNIE ZAMÓWIĆ!</t>
+  </si>
+  <si>
+    <t>Nie ma w mouser</t>
+  </si>
+  <si>
+    <t xml:space="preserve">667-EEF-CX0J101R </t>
+  </si>
+  <si>
+    <t>80-C0805C106M8RAUTLR</t>
+  </si>
+  <si>
+    <t>Kondensator 10uF 10V 0805</t>
+  </si>
+  <si>
+    <t>GRM21BR60J107ME15L</t>
+  </si>
+  <si>
+    <t>100nF 0805</t>
   </si>
 </sst>
 </file>
@@ -1609,24 +1676,6 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1649,6 +1698,24 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2002,7 +2069,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.28515625" style="4" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
     <col min="3" max="3" width="21.28515625" customWidth="1"/>
     <col min="4" max="4" width="33.7109375" customWidth="1"/>
     <col min="5" max="5" width="34.7109375" customWidth="1"/>
@@ -2016,45 +2083,45 @@
     <col min="13" max="13" width="9.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="106" t="s">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A1" s="100" t="s">
         <v>207</v>
       </c>
-      <c r="B1" s="104" t="s">
+      <c r="B1" s="98" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="102" t="s">
+      <c r="C1" s="110" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="102" t="s">
+      <c r="D1" s="110" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="102" t="s">
+      <c r="E1" s="110" t="s">
         <v>99</v>
       </c>
-      <c r="F1" s="100" t="s">
+      <c r="F1" s="108" t="s">
         <v>120</v>
       </c>
-      <c r="G1" s="108" t="s">
+      <c r="G1" s="102" t="s">
         <v>132</v>
       </c>
-      <c r="H1" s="109"/>
-      <c r="I1" s="110" t="s">
+      <c r="H1" s="103"/>
+      <c r="I1" s="104" t="s">
         <v>134</v>
       </c>
-      <c r="J1" s="111"/>
-      <c r="K1" s="98" t="s">
+      <c r="J1" s="105"/>
+      <c r="K1" s="106" t="s">
         <v>133</v>
       </c>
-      <c r="L1" s="99"/>
-    </row>
-    <row r="2" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="107"/>
-      <c r="B2" s="105"/>
-      <c r="C2" s="103"/>
-      <c r="D2" s="103"/>
-      <c r="E2" s="103"/>
-      <c r="F2" s="101"/>
+      <c r="L1" s="107"/>
+    </row>
+    <row r="2" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="101"/>
+      <c r="B2" s="99"/>
+      <c r="C2" s="111"/>
+      <c r="D2" s="111"/>
+      <c r="E2" s="111"/>
+      <c r="F2" s="109"/>
       <c r="G2" s="50" t="s">
         <v>121</v>
       </c>
@@ -2077,7 +2144,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="28">
         <v>4</v>
       </c>
@@ -2114,7 +2181,7 @@
         <v>1.6459800000000002</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>1</v>
       </c>
@@ -2147,7 +2214,7 @@
         <v>2.4576000000000002</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>1</v>
       </c>
@@ -2180,7 +2247,7 @@
         <v>2.1852</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>1</v>
       </c>
@@ -2212,8 +2279,11 @@
         <f t="shared" si="0"/>
         <v>1.7052</v>
       </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O6" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>1</v>
       </c>
@@ -2246,7 +2316,7 @@
         <v>0.50004000000000004</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>4</v>
       </c>
@@ -2278,8 +2348,11 @@
         <f t="shared" si="0"/>
         <v>11.852399999999999</v>
       </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O8" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>3</v>
       </c>
@@ -2312,7 +2385,7 @@
         <v>3.3119999999999998</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>4</v>
       </c>
@@ -2345,7 +2418,7 @@
         <v>3.9050000000000002</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>2</v>
       </c>
@@ -2378,7 +2451,7 @@
         <v>1.7569999999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>1</v>
       </c>
@@ -2411,7 +2484,7 @@
         <v>3.6560000000000001</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>1</v>
       </c>
@@ -2444,7 +2517,7 @@
         <v>2.5872000000000002</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>1</v>
       </c>
@@ -2477,7 +2550,7 @@
         <v>5.9390000000000001</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>1</v>
       </c>
@@ -2510,7 +2583,7 @@
         <v>6.7129999999999992</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>1</v>
       </c>
@@ -2764,6 +2837,9 @@
       </c>
       <c r="L24" s="49" t="s">
         <v>215</v>
+      </c>
+      <c r="M24" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="25" spans="1:29" x14ac:dyDescent="0.25">
@@ -3530,6 +3606,7 @@
     <hyperlink ref="L18" r:id="rId40" xr:uid="{09BA8893-4495-41E7-88F8-697E23A9411C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId41"/>
 </worksheet>
 </file>
 
@@ -3554,39 +3631,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A1" s="106" t="s">
+      <c r="A1" s="100" t="s">
         <v>207</v>
       </c>
-      <c r="B1" s="104" t="s">
+      <c r="B1" s="98" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="102" t="s">
+      <c r="C1" s="110" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="102" t="s">
+      <c r="D1" s="110" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="102" t="s">
+      <c r="E1" s="110" t="s">
         <v>99</v>
       </c>
-      <c r="F1" s="100" t="s">
+      <c r="F1" s="108" t="s">
         <v>120</v>
       </c>
-      <c r="G1" s="108" t="s">
+      <c r="G1" s="102" t="s">
         <v>132</v>
       </c>
       <c r="H1" s="112"/>
-      <c r="I1" s="110" t="s">
+      <c r="I1" s="104" t="s">
         <v>134</v>
       </c>
-      <c r="J1" s="111"/>
-      <c r="K1" s="98" t="s">
+      <c r="J1" s="105"/>
+      <c r="K1" s="106" t="s">
         <v>133</v>
       </c>
-      <c r="L1" s="99"/>
+      <c r="L1" s="107"/>
     </row>
     <row r="2" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="107"/>
+      <c r="A2" s="101"/>
       <c r="B2" s="113"/>
       <c r="C2" s="114"/>
       <c r="D2" s="114"/>
@@ -5343,4 +5420,158 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5673A395-CBE6-40D4-87FC-F1A8F9554773}">
+  <dimension ref="A2:F10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="37.85546875" customWidth="1"/>
+    <col min="2" max="2" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.5703125" customWidth="1"/>
+    <col min="4" max="4" width="38.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>261</v>
+      </c>
+      <c r="C2" t="s">
+        <v>265</v>
+      </c>
+      <c r="D2" t="s">
+        <v>260</v>
+      </c>
+      <c r="E2" t="s">
+        <v>266</v>
+      </c>
+      <c r="F2" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>255</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>268</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>256</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4" s="73" t="s">
+        <v>263</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>257</v>
+      </c>
+      <c r="B5">
+        <v>20</v>
+      </c>
+      <c r="C5" s="73" t="s">
+        <v>264</v>
+      </c>
+      <c r="D5">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>258</v>
+      </c>
+      <c r="B6">
+        <v>20</v>
+      </c>
+      <c r="C6" s="73" t="s">
+        <v>241</v>
+      </c>
+      <c r="D6">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>259</v>
+      </c>
+      <c r="B7">
+        <v>20</v>
+      </c>
+      <c r="C7" s="73" t="s">
+        <v>269</v>
+      </c>
+      <c r="D7">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>262</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" s="73" t="s">
+        <v>187</v>
+      </c>
+      <c r="D8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>271</v>
+      </c>
+      <c r="B9">
+        <v>15</v>
+      </c>
+      <c r="C9" s="73" t="s">
+        <v>270</v>
+      </c>
+      <c r="D9">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>273</v>
+      </c>
+      <c r="B10">
+        <v>15</v>
+      </c>
+      <c r="C10" s="73" t="s">
+        <v>272</v>
+      </c>
+      <c r="D10">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C5" r:id="rId1" display="https://www.mouser.pl/ProductDetail/Molex/46765-0301?qs=bpeZmj96Seed20dZhMSXqw%3D%3D" xr:uid="{073EBA41-AC5A-40F9-8363-2E27B7386BCD}"/>
+    <hyperlink ref="C4" r:id="rId2" display="https://www.mouser.pl/ProductDetail/Raspberry-Pi/SC0358?qs=sGAEpiMZZMsvnOgGvSjZeHfx0dldyM%2Fty40t4MMDEBqB8FZUAXZoPQ%3D%3D" xr:uid="{C4019E9A-1E3A-40BD-B842-BE6180D7E352}"/>
+    <hyperlink ref="C6" r:id="rId3" xr:uid="{43E18FEA-033F-46EC-A684-A32250D00792}"/>
+    <hyperlink ref="C7" r:id="rId4" xr:uid="{A2F2DD76-8F39-45B7-9B8C-DFF6651F71D7}"/>
+    <hyperlink ref="C8" r:id="rId5" xr:uid="{71C3B908-2430-4BDC-ACF3-C948C9CFFF4A}"/>
+    <hyperlink ref="C9" r:id="rId6" xr:uid="{D155872E-3D18-42CD-ADEF-3340CF9476F6}"/>
+    <hyperlink ref="C10" r:id="rId7" xr:uid="{322E6D2C-5234-40B8-8936-7C647FDB3076}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
remove unnecessary files, update BOM
</commit_message>
<xml_diff>
--- a/CM5IO_BOM.xlsx
+++ b/CM5IO_BOM.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Elektronika Schematy\KiCad\IARC-RPi_CM5_drone_platform\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Elektronika Schematy\KiCad\IARC-RPi_CM_Drone_Board\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD108B92-E698-4CEB-89CB-2782784DAF2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5624364-F3A0-4C0A-B5C5-254C646C17AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" activeTab="4" xr2:uid="{2D0DF511-CD42-495F-98C8-D8FF06CCC30B}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{2D0DF511-CD42-495F-98C8-D8FF06CCC30B}"/>
   </bookViews>
   <sheets>
     <sheet name="Bottom" sheetId="1" r:id="rId1"/>

</xml_diff>